<commit_message>
Updates SYAHPC to align with BIFU
</commit_message>
<xml_diff>
--- a/InputData/hydgn/SYAHPC/Start Year Annual Hydrogen Production Capacity.xlsx
+++ b/InputData/hydgn/SYAHPC/Start Year Annual Hydrogen Production Capacity.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\hydgn\SYAHPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA4422A-02F3-4889-8B7D-04E7528453DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6577AB45-5DF6-45E7-9726-5FF98A55CA3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="1815" windowWidth="21600" windowHeight="12585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="SYAHPC" sheetId="5" r:id="rId2"/>
+    <sheet name="BIFU" sheetId="6" r:id="rId2"/>
+    <sheet name="SYAHPC" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="btu_per_kwh">#REF!</definedName>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Source:</t>
   </si>
@@ -83,26 +84,137 @@
     <t>This variable should be equal to the total start year hydrogen fuel demand from BIFU</t>
   </si>
   <si>
-    <t>FILL OUT</t>
-  </si>
-  <si>
     <t xml:space="preserve"> (or higher if current production facilities are running under max capacity)</t>
   </si>
   <si>
-    <t>SYAHPC Start Year Annual Green Hydrogen Production Capacity</t>
-  </si>
-  <si>
-    <t>SYAHPC Start Year Annual Low Carbon Hydrogen Production Capacity</t>
-  </si>
-  <si>
-    <t>SYAHPC Start Year Annual Unspecified Hydrogen Production Capacity</t>
+    <t>Unit: BTU</t>
+  </si>
+  <si>
+    <t>agriculture and forestry 01T03</t>
+  </si>
+  <si>
+    <t>coal mining 05</t>
+  </si>
+  <si>
+    <t>oil and gas extraction 06</t>
+  </si>
+  <si>
+    <t>other mining and quarrying 07T08</t>
+  </si>
+  <si>
+    <t>food beverage and tobacco 10T12</t>
+  </si>
+  <si>
+    <t>textiles apparel and leather 13T15</t>
+  </si>
+  <si>
+    <t>wood products 16</t>
+  </si>
+  <si>
+    <t>pulp paper and printing 17T18</t>
+  </si>
+  <si>
+    <t>refined petroleum and coke 19</t>
+  </si>
+  <si>
+    <t>chemicals 20</t>
+  </si>
+  <si>
+    <t>rubber and plastic products 22</t>
+  </si>
+  <si>
+    <t>glass and glass products 231</t>
+  </si>
+  <si>
+    <t>cement and other nonmetallic minerals 239</t>
+  </si>
+  <si>
+    <t>iron and steel 241</t>
+  </si>
+  <si>
+    <t>other metals 242</t>
+  </si>
+  <si>
+    <t>metal products except machinery and vehicles 25</t>
+  </si>
+  <si>
+    <t>computers and electronics 26</t>
+  </si>
+  <si>
+    <t>appliances and electrical equipment 27</t>
+  </si>
+  <si>
+    <t>other machinery 28</t>
+  </si>
+  <si>
+    <t>road vehicles 29</t>
+  </si>
+  <si>
+    <t>nonroad vehicles 30</t>
+  </si>
+  <si>
+    <t>other manufacturing 31T33</t>
+  </si>
+  <si>
+    <t>energy pipelines and gas processing 352T353</t>
+  </si>
+  <si>
+    <t>water and waste 36T39</t>
+  </si>
+  <si>
+    <t>construction 41T43</t>
+  </si>
+  <si>
+    <t>Time (Year)</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[transportation sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[electricity sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[residential buildings sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[commercial buildings sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[industry sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[district heat and hydrogen sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[LULUCF sector] : test</t>
+  </si>
+  <si>
+    <t>BAU Total Hydrogen Demand by Sector[geoengineering sector] : test</t>
+  </si>
+  <si>
+    <t>Production shares by tech</t>
+  </si>
+  <si>
+    <t>Energy Futures Initiative</t>
+  </si>
+  <si>
+    <t>The U.S. Hydrogen Demand Action Plan</t>
+  </si>
+  <si>
+    <t>https://energyfuturesinitiative.org/wp-content/uploads/sites/2/2023/02/EFI-Hydrogen-Hubs-FINAL-2-1.pdf</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>SYAHPC Start Year Annual Hydrogen Production Capacity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,6 +238,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -136,7 +255,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -160,12 +279,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -182,6 +301,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>437079</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>115454</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>211674</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>162427</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E96FBAC0-03AD-4649-9E01-F860DE0D7D8A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2267858" y="296883"/>
+          <a:ext cx="4656673" cy="2949830"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,138 +616,447 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="45.85546875" customWidth="1"/>
+    <col min="2" max="2" width="45.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B8" s="3"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="1"/>
+      <c r="B5" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B7" s="2">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B9" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B9" r:id="rId1" xr:uid="{3D4A8A29-B2AD-419F-8725-FF93E29DE553}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49F6B76C-DFC9-455B-973C-BACABC36BDD5}">
+  <dimension ref="B2:C37"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7">
+        <v>673817381738.17383</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11">
+        <v>483583466000000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12">
+        <v>238311560322698.94</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19">
+        <v>3503850385038.5039</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B23" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="4">
+        <v>507088000000</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B34" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="4">
+        <v>726078000000000</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B35" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B36" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B37" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B86B67DC-846A-43A5-93A4-7633904409D9}">
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5">
-        <v>39900000000000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B2" s="4">
+        <f>0.5*BIFU!$C$30</f>
+        <v>253544000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5">
-        <v>759000000000000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B3" s="4">
+        <f>0.5*BIFU!$C$30+BIFU!C34</f>
+        <v>726331544000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B5" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B6" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>